<commit_message>
sync da monorepo @eed409b (SAL rework + pptx + Excel)
</commit_message>
<xml_diff>
--- a/DOCS/piani/Logistico2.0_Piano_Attivita_Gantt.xlsx
+++ b/DOCS/piani/Logistico2.0_Piano_Attivita_Gantt.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,8 +74,16 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -130,6 +138,11 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000E5A63"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -157,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -222,6 +235,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4287,8 +4307,8 @@
     <mergeCell ref="Y2:AC2"/>
     <mergeCell ref="U2:X2"/>
     <mergeCell ref="AH2:AK2"/>
+    <mergeCell ref="A47:AK47"/>
     <mergeCell ref="A23:AK23"/>
-    <mergeCell ref="A47:AK47"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="A1:AK1"/>
     <mergeCell ref="AD2:AG2"/>
@@ -4305,7 +4325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4318,6 +4338,7 @@
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -4386,6 +4407,11 @@
       <c r="J3" s="4" t="inlineStr">
         <is>
           <t>DIC</t>
+        </is>
+      </c>
+      <c r="K3" s="24" t="inlineStr">
+        <is>
+          <t>STATO (27/08/2026)</t>
         </is>
       </c>
     </row>
@@ -4432,6 +4458,11 @@
       <c r="H5" s="12" t="n"/>
       <c r="I5" s="12" t="n"/>
       <c r="J5" s="12" t="n"/>
+      <c r="K5" s="25" t="inlineStr">
+        <is>
+          <t>Infra su GitLab; terraform plan DEV ✅, apply in attesa grant UC alla MI (OP-INF-1)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
@@ -4454,6 +4485,11 @@
       <c r="H6" s="13" t="n"/>
       <c r="I6" s="12" t="n"/>
       <c r="J6" s="12" t="n"/>
+      <c r="K6" s="25" t="inlineStr">
+        <is>
+          <t>DIM sviluppate; first-run su cloud da avviare</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
@@ -4476,6 +4512,11 @@
       <c r="H7" s="10" t="n"/>
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="12" t="n"/>
+      <c r="K7" s="25" t="inlineStr">
+        <is>
+          <t>Carichi sviluppati (orphan 0,0%); quadratura vs Oracle + BA su cloud</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
@@ -4498,6 +4539,11 @@
       <c r="H8" s="13" t="n"/>
       <c r="I8" s="13" t="n"/>
       <c r="J8" s="12" t="n"/>
+      <c r="K8" s="25" t="inlineStr">
+        <is>
+          <t>Giacenze sviluppate; quadratura + backfill su cloud</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
@@ -4520,6 +4566,11 @@
       <c r="H9" s="10" t="n"/>
       <c r="I9" s="10" t="n"/>
       <c r="J9" s="12" t="n"/>
+      <c r="K9" s="25" t="inlineStr">
+        <is>
+          <t>Prep. Spedizioni sviluppate; quadratura + edge-case + BA su cloud</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
@@ -4542,6 +4593,11 @@
       <c r="H10" s="10" t="n"/>
       <c r="I10" s="10" t="n"/>
       <c r="J10" s="12" t="n"/>
+      <c r="K10" s="25" t="inlineStr">
+        <is>
+          <t>Trasporti sviluppati; quadratura su cloud (listini corrieri assenti)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
@@ -4564,6 +4620,11 @@
       <c r="H11" s="10" t="n"/>
       <c r="I11" s="10" t="n"/>
       <c r="J11" s="12" t="n"/>
+      <c r="K11" s="25" t="inlineStr">
+        <is>
+          <t>CE178 + carrellisti sviluppati; validazione funzionale su cloud</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
@@ -4586,6 +4647,11 @@
       <c r="H12" s="10" t="n"/>
       <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
+      <c r="K12" s="25" t="inlineStr">
+        <is>
+          <t>Aggregati/KPI sviluppati; MicroStrategy + tuning su cloud</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
@@ -4608,6 +4674,11 @@
       <c r="H13" s="14" t="n"/>
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="n"/>
+      <c r="K13" s="25" t="inlineStr">
+        <is>
+          <t>Shadow/cut-over: bozze; bloccato su provisioning PROD</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -4627,6 +4698,13 @@
       <c r="H14" s="21" t="n"/>
       <c r="I14" s="21" t="n"/>
       <c r="J14" s="21" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>Nota SAL 27/08/2026: barre = piano di sviluppo (build). Validazione cloud/go-live per wave: SET26→FEB27 (target).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="22" t="inlineStr">
@@ -7044,9 +7122,9 @@
   <mergeCells count="11">
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A51:I51"/>
-    <mergeCell ref="A5:I5"/>
     <mergeCell ref="A28:I28"/>
     <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A5:I5"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A40:I40"/>

</xml_diff>